<commit_message>
Agrega pipeline fold-safe y actualiza documentación de modelado
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="1" r:id="R43c675938d144e83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="Rbda25b36bcf34e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="1" r:id="R9467ee7873f34205"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="R7a22692f5ae040d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BitacoraTable" displayName="BitacoraTable" ref="A1:L17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BitacoraTable" displayName="BitacoraTable" ref="A1:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Fecha"/>
@@ -106,7 +106,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoadmapTable" displayName="RoadmapTable" ref="A1:F12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoadmapTable" displayName="RoadmapTable" ref="A1:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Orden"/>
     <x:tableColumn id="2" name="Etapa"/>
@@ -813,7 +813,7 @@
         <x:v>Implementar pipeline fold-safe obligatorio para CV final.</x:v>
       </x:c>
       <x:c r="J13" s="12" t="str">
-        <x:v>Planeado</x:v>
+        <x:v>Cerrado</x:v>
       </x:c>
       <x:c r="K13" s="12" t="str">
         <x:v>Sí</x:v>
@@ -1010,6 +1010,158 @@
       </x:c>
       <x:c r="L18" s="12" t="str">
         <x:v>03_stuff_baseline.py</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A19" s="12" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>04_fold_safe_arsenal.py</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>Cierre de arsenal fold-safe</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
+        <x:v>Construcción leakage-safe de referencias y features específicas del pitcher.</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="str">
+        <x:v>Pitcher holdout y season-forward temporal: 2024 a 2025; 2024–2025 a 2026.</x:v>
+      </x:c>
+      <x:c r="G19" s="12" t="str">
+        <x:v>Unseen: 0% de cobertura por diseño. Cohorte con historial: 96.2% en 2025 y 98.0% en 2026.</x:v>
+      </x:c>
+      <x:c r="H19" s="12" t="str">
+        <x:v>FB histórica disponible: 132,886/138,110 (2025); 88,409/90,176 (2026). Leakage: PASS.</x:v>
+      </x:c>
+      <x:c r="I19" s="12" t="str">
+        <x:v>Unseen pitcher: Physical Stuff. Known pitcher / future season: Physical Stuff + Historical Arsenal. Sin fallback.</x:v>
+      </x:c>
+      <x:c r="J19" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K19" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L19" s="12" t="str">
+        <x:v>04_fold_safe_arsenal.py; 04_fold_safe_arsenal_audit.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A20" s="12" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="str">
+        <x:v>04_fold_safe_arsenal.py</x:v>
+      </x:c>
+      <x:c r="D20" s="12" t="str">
+        <x:v>Primary fastball determinística</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="str">
+        <x:v>Resolver empates sin depender del orden de filas.</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="str">
+        <x:v>Four-Seam/Sinker por mayor uso; empate: mayor mean RelSpeed del periodo permitido; empate final: Four-Seam.</x:v>
+      </x:c>
+      <x:c r="G20" s="12" t="str">
+        <x:v>Velocidad válida precede a NaN; ambas NaN: Four-Seam. No se imputan velocidades.</x:v>
+      </x:c>
+      <x:c r="H20" s="12" t="str">
+        <x:v>Mínimo 20 pitches. Determinismo con filas invertidas y barajadas: PASS.</x:v>
+      </x:c>
+      <x:c r="I20" s="12" t="str">
+        <x:v>El tie-break de velocidad utiliza solo el fold o historial previo permitido.</x:v>
+      </x:c>
+      <x:c r="J20" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K20" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L20" s="12" t="str">
+        <x:v>04_fold_safe_arsenal.py; 04_fold_safe_arsenal_audit.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A21" s="12" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="str">
+        <x:v>04_fold_safe_arsenal.py</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="str">
+        <x:v>Estabilidad temporal</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="str">
+        <x:v>¿Son permanentes la primary fastball y la composición del arsenal?</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="str">
+        <x:v>Auditoría descriptiva posterior; ninguna estadística futura se utiliza como feature.</x:v>
+      </x:c>
+      <x:c r="G21" s="12" t="str">
+        <x:v>Primary FB estable: 91.16% (2024 a 2025) y 88.98% (2025 a 2026). Usage cambia moderadamente.</x:v>
+      </x:c>
+      <x:c r="H21" s="12" t="str">
+        <x:v>Usage: cambio absoluto medio 6.4775 pp y 6.7860 pp. Pares comparables, sin ponderación.</x:v>
+      </x:c>
+      <x:c r="I21" s="12" t="str">
+        <x:v>Actualizar las referencias temporalmente; no definir propiedades permanentes para toda la carrera.</x:v>
+      </x:c>
+      <x:c r="J21" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K21" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L21" s="12" t="str">
+        <x:v>04_primary_fastball_changes.csv; 04_fold_safe_arsenal_audit.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A22" s="12" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C22" s="12" t="str">
+        <x:v>05_arsenal_incremental_value.py</x:v>
+      </x:c>
+      <x:c r="D22" s="12" t="str">
+        <x:v>Próximo paso</x:v>
+      </x:c>
+      <x:c r="E22" s="12" t="str">
+        <x:v>Medir valor incremental del arsenal histórico sobre Physical Stuff para is_whiff usando exactamente las mismas filas elegibles.</x:v>
+      </x:c>
+      <x:c r="F22" s="12" t="str">
+        <x:v>Comparación futura en ventanas season-forward con historial previo permitido.</x:v>
+      </x:c>
+      <x:c r="G22" s="12" t="str">
+        <x:v>Pendiente. No se entrenaron modelos ni se demostró mejora predictiva del arsenal en 04.</x:v>
+      </x:c>
+      <x:c r="H22" s="12" t="str">
+        <x:v>Sin resultados de 05.</x:v>
+      </x:c>
+      <x:c r="I22" s="12" t="str">
+        <x:v>Siguiente paso vigente. La tarea previa 05_target_definitions se conserva pendiente para los targets derivados.</x:v>
+      </x:c>
+      <x:c r="J22" s="12" t="str">
+        <x:v>Planeado</x:v>
+      </x:c>
+      <x:c r="K22" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L22" s="12" t="str">
+        <x:v>05_arsenal_incremental_value.py (por crear)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1023,7 +1175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0360408c24d54620"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbabd1c52f7a144b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1134,7 +1286,7 @@
         <x:v>Eliminar leakage de features agregadas.</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>Siguiente</x:v>
+        <x:v>Cerrado</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
         <x:v>Pipeline fold-safe de arsenal para medir valor incremental sin leakage.</x:v>
@@ -1278,6 +1430,26 @@
       </x:c>
       <x:c r="F12" s="12" t="str">
         <x:v>Entregable final.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A13" s="12" t="n">
+        <x:v>4.5</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="str">
+        <x:v>Valor incremental de arsenal</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="str">
+        <x:v>05_arsenal_incremental_value.py</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="str">
+        <x:v>Medir valor incremental sobre Physical Stuff para is_whiff usando exactamente las mismas filas elegibles.</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="str">
+        <x:v>Siguiente</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="str">
+        <x:v>Determinar si el arsenal añade señal. Sin resultado anticipado; targets derivados siguen pendientes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1288,7 +1460,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R589f24d4207a4863"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reda8033ae6c34c3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Definiciones de targets y explicacion facil
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="1" r:id="R9467ee7873f34205"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="R7a22692f5ae040d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bitácora" sheetId="1" r:id="R8a4257dc67984663"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" r:id="R5efb21104bdf444d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BitacoraTable" displayName="BitacoraTable" ref="A1:L22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BitacoraTable" displayName="BitacoraTable" ref="A1:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Fecha"/>
@@ -830,7 +830,7 @@
         <x:v>2026-09-09</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>05_target_definitions</x:v>
+        <x:v>05_target_definitions.py</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
         <x:v>Targets derivados</x:v>
@@ -851,7 +851,7 @@
         <x:v>Crear documento de definiciones antes de entrenar esos targets.</x:v>
       </x:c>
       <x:c r="J14" s="12" t="str">
-        <x:v>Planeado</x:v>
+        <x:v>Cerrado</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str">
         <x:v>Sí</x:v>
@@ -1126,7 +1126,7 @@
         <x:v>04_primary_fastball_changes.csv; 04_fold_safe_arsenal_audit.txt</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="22" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A22" s="12" t="n">
         <x:v>21</x:v>
       </x:c>
@@ -1152,7 +1152,7 @@
         <x:v>Sin resultados de 05.</x:v>
       </x:c>
       <x:c r="I22" s="12" t="str">
-        <x:v>Siguiente paso vigente. La tarea previa 05_target_definitions se conserva pendiente para los targets derivados.</x:v>
+        <x:v>Experimento pendiente. Actualización 24/09/2026: primero revisar 05_target_definitions.py; no entrenar aún.</x:v>
       </x:c>
       <x:c r="J22" s="12" t="str">
         <x:v>Planeado</x:v>
@@ -1162,6 +1162,272 @@
       </x:c>
       <x:c r="L22" s="12" t="str">
         <x:v>05_arsenal_incremental_value.py (por crear)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A23" s="12" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B23" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C23" s="12" t="str">
+        <x:v>05_target_definitions.py</x:v>
+      </x:c>
+      <x:c r="D23" s="12" t="str">
+        <x:v>Auditoría real de targets</x:v>
+      </x:c>
+      <x:c r="E23" s="12" t="str">
+        <x:v>Revisar disponibilidad, categorías y denominadores antes de fijar targets V1.</x:v>
+      </x:c>
+      <x:c r="F23" s="12" t="str">
+        <x:v>Dataset original completo, sin filtros V1; 635,002 filas y 84 columnas.</x:v>
+      </x:c>
+      <x:c r="G23" s="12" t="str">
+        <x:v>26/26 columnas disponibles; 18 flags binarios sin NaN ni valores inválidos.</x:v>
+      </x:c>
+      <x:c r="H23" s="12" t="str">
+        <x:v>Whiff/pitch: 71,914/635,002 = 11.3250%; whiff/swing: 71,914/298,029 = 24.1299%; chase/outside: 141,014/411,912 = 34.2340%.</x:v>
+      </x:c>
+      <x:c r="I23" s="12" t="str">
+        <x:v>Auditoría ejecutada. Definiciones pendientes de revisión conjunta; 05 no cerrado. Sin entrenamiento.</x:v>
+      </x:c>
+      <x:c r="J23" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K23" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L23" s="12" t="str">
+        <x:v>05_target_definitions_audit.txt; stuff_model_df.parquet</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A24" s="12" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B24" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C24" s="12" t="str">
+        <x:v>05_target_definitions.py</x:v>
+      </x:c>
+      <x:c r="D24" s="12" t="str">
+        <x:v>Consistencia y semántica</x:v>
+      </x:c>
+      <x:c r="E24" s="12" t="str">
+        <x:v>¿Coinciden los flags con las categorías reales?</x:v>
+      </x:c>
+      <x:c r="F24" s="12" t="str">
+        <x:v>Comparaciones de flags y cruces con PitchCall, KorBB y play_result.</x:v>
+      </x:c>
+      <x:c r="G24" s="12" t="str">
+        <x:v>403 called strikes con swing; 450 whiff con contact; is_hit_by_pitch siempre 0 pese a 2,280 HitByPitch en PitchCall (2,258 en play_result).</x:v>
+      </x:c>
+      <x:c r="H24" s="12" t="str">
+        <x:v>0 diferencias whiff/swinging strike; 0 whiff o contact sin swing; 0 chase dentro de zona. is_batted incluye fouls.</x:v>
+      </x:c>
+      <x:c r="I24" s="12" t="str">
+        <x:v>Whiff, hit, strikeout y walk parecen directos según cruces; called strike y swing/contact requieren revisar contradicciones. No recodificar silenciosamente.</x:v>
+      </x:c>
+      <x:c r="J24" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K24" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L24" s="12" t="str">
+        <x:v>05_target_definitions_audit.txt, secciones D y L</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A25" s="12" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C25" s="12" t="str">
+        <x:v>05_target_definitions.py</x:v>
+      </x:c>
+      <x:c r="D25" s="12" t="str">
+        <x:v>Contacto y targets abiertos</x:v>
+      </x:c>
+      <x:c r="E25" s="12" t="str">
+        <x:v>¿Qué permite definir hit_type y qué evidencia falta?</x:v>
+      </x:c>
+      <x:c r="F25" s="12" t="str">
+        <x:v>225,722 is_batted=1; distribuciones de hit_type, ExitSpeed, Angle y resultados.</x:v>
+      </x:c>
+      <x:c r="G25" s="12" t="str">
+        <x:v>GroundBall: 63,890; hit_type ausente: 41,685 (18.47%). ExitSpeed ausente: 42,901; Angle: 42,902.</x:v>
+      </x:c>
+      <x:c r="H25" s="12" t="str">
+        <x:v>GroundBall Angle media -13.283°, mediana -7.273°. ExitSpeed: media 79.851 mph, rango 1.140–129.918.</x:v>
+      </x:c>
+      <x:c r="I25" s="12" t="str">
+        <x:v>Groundball candidato derivable, sin tratar ausentes como negativos. Weak/hard contact y out-within-PA abiertos. xRunValue no construido; sin pesos externos.</x:v>
+      </x:c>
+      <x:c r="J25" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K25" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L25" s="12" t="str">
+        <x:v>05_target_definitions_audit.txt, secciones G–K</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A26" s="12" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C26" s="12" t="str">
+        <x:v>05_target_definitions.py</x:v>
+      </x:c>
+      <x:c r="D26" s="12" t="str">
+        <x:v>Prioridad vigente y validación</x:v>
+      </x:c>
+      <x:c r="E26" s="12" t="str">
+        <x:v>Auditar targets antes de continuar con experimentos de modelado.</x:v>
+      </x:c>
+      <x:c r="F26" s="12" t="str">
+        <x:v>Ejecución completa y 4 pruebas de robustez: faltantes/vacío, NaN, tipos/categorías inesperados, denominador cero.</x:v>
+      </x:c>
+      <x:c r="G26" s="12" t="str">
+        <x:v>Ejecución correcta y pruebas PASS. Datos originales intactos. Avisos de PyArrow al consultar caché CPU bajo sandbox, sin fallo de lectura.</x:v>
+      </x:c>
+      <x:c r="H26" s="12" t="str">
+        <x:v>Resumen TXT reproducible con SHA256 del dataset y versiones de Python/pandas/NumPy.</x:v>
+      </x:c>
+      <x:c r="I26" s="12" t="str">
+        <x:v>Revisar anomalías y acordar targets. El experimento incremental de arsenal permanece pendiente; no avanzar todavía.</x:v>
+      </x:c>
+      <x:c r="J26" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K26" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L26" s="12" t="str">
+        <x:v>05_target_definitions.py; 05_target_definitions_audit.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A27" s="12" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C27" s="12" t="str">
+        <x:v>05_target_definitions.py</x:v>
+      </x:c>
+      <x:c r="D27" s="12" t="str">
+        <x:v>Cierre formal V1</x:v>
+      </x:c>
+      <x:c r="E27" s="12" t="str">
+        <x:v>Ratificar fuentes y universos elegibles.</x:v>
+      </x:c>
+      <x:c r="F27" s="12" t="str">
+        <x:v>Auditorías de flags, anomalías, BIP/contacto y estructura PA.</x:v>
+      </x:c>
+      <x:c r="G27" s="12" t="str">
+        <x:v>Incluidos: whiff/pitch; whiff/swing; called strike desde PitchCall; chase/outside; groundball en BIP conocido no-bunt.</x:v>
+      </x:c>
+      <x:c r="H27" s="12" t="str">
+        <x:v>GB: 49,103/107,118 = 45.8401%; cobertura BIP 92.3845%. Contacto medido: 107,117.</x:v>
+      </x:c>
+      <x:c r="I27" s="12" t="str">
+        <x:v>Fuera V1: weak/hard contact, out-within-PA, xRunValue. No usar is_hit_by_pitch. Contradicciones conservadas.</x:v>
+      </x:c>
+      <x:c r="J27" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K27" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L27" s="12" t="str">
+        <x:v>05_target_definitions_audit.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A28" s="12" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B28" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C28" s="12" t="str">
+        <x:v>05_target_definitions.py</x:v>
+      </x:c>
+      <x:c r="D28" s="12" t="str">
+        <x:v>Justificación técnica</x:v>
+      </x:c>
+      <x:c r="E28" s="12" t="str">
+        <x:v>No introducir convenciones arbitrarias ni corregir sin procedencia.</x:v>
+      </x:c>
+      <x:c r="F28" s="12" t="str">
+        <x:v>403 called strike+contact; 450 whiff+contact; 22 HBP con resultado Walk.</x:v>
+      </x:c>
+      <x:c r="G28" s="12" t="str">
+        <x:v>is_batted no equivale a BIP. hit_type/Angle muestran cortes cerca de 10/25/50 grados; procedencia no confirmada.</x:v>
+      </x:c>
+      <x:c r="H28" s="12" t="str">
+        <x:v>6,549 BIP sin hit_type ni mediciones; 2,281 bunts excluidos. Sin identificador/orden PA validado; 325 UUID v4.</x:v>
+      </x:c>
+      <x:c r="I28" s="12" t="str">
+        <x:v>PitchCall gobierna called strike sin eliminar contradicciones. No usar hit_type y Angle como validación independiente.</x:v>
+      </x:c>
+      <x:c r="J28" s="12" t="str">
+        <x:v>Cerrado</x:v>
+      </x:c>
+      <x:c r="K28" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L28" s="12" t="str">
+        <x:v>05_target_definitions_audit.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A29" s="12" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B29" s="12" t="str">
+        <x:v>2026-09-24</x:v>
+      </x:c>
+      <x:c r="C29" s="12" t="str">
+        <x:v>06_arsenal_incremental_value.py</x:v>
+      </x:c>
+      <x:c r="D29" s="12" t="str">
+        <x:v>Siguiente paso</x:v>
+      </x:c>
+      <x:c r="E29" s="12" t="str">
+        <x:v>¿Añade valor predictivo el arsenal histórico?</x:v>
+      </x:c>
+      <x:c r="F29" s="12" t="str">
+        <x:v>Null vs Physical Stuff vs Physical Stuff + Historical Arsenal; is_whiff.</x:v>
+      </x:c>
+      <x:c r="G29" s="12" t="str">
+        <x:v>Pendiente: no hay resultados ni entrenamiento de 06.</x:v>
+      </x:c>
+      <x:c r="H29" s="12" t="str">
+        <x:v>Mismas filas elegibles season-forward para las tres alternativas.</x:v>
+      </x:c>
+      <x:c r="I29" s="12" t="str">
+        <x:v>Retomar experimento pospuesto, ahora numerado 06. No anticipar mejora.</x:v>
+      </x:c>
+      <x:c r="J29" s="12" t="str">
+        <x:v>Planeado</x:v>
+      </x:c>
+      <x:c r="K29" s="12" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="L29" s="12" t="str">
+        <x:v>06_arsenal_incremental_value.py (por crear)</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1175,7 +1441,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbabd1c52f7a144b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cc50f9d3d9a4433"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1292,7 +1558,7 @@
         <x:v>Pipeline fold-safe de arsenal para medir valor incremental sin leakage.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -1300,16 +1566,16 @@
         <x:v>Targets derivados</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>05_target_definitions</x:v>
+        <x:v>05_target_definitions.py</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
         <x:v>Formalizar groundball, weak/hard contact y xRunValue.</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>Planeado</x:v>
+        <x:v>Cerrado</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>Targets reproducibles y auditables.</x:v>
+        <x:v>Targets V1 ratificados; ver cierre en bitácora. Sin corrección de etiquetas.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1432,7 +1698,7 @@
         <x:v>Entregable final.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A13" s="12" t="n">
         <x:v>4.5</x:v>
       </x:c>
@@ -1440,16 +1706,16 @@
         <x:v>Valor incremental de arsenal</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>05_arsenal_incremental_value.py</x:v>
+        <x:v>06_arsenal_incremental_value.py</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
-        <x:v>Medir valor incremental sobre Physical Stuff para is_whiff usando exactamente las mismas filas elegibles.</x:v>
+        <x:v>Comparar Null, Physical Stuff y Physical Stuff + Historical Arsenal para is_whiff sobre las mismas filas elegibles season-forward.</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
         <x:v>Siguiente</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
-        <x:v>Determinar si el arsenal añade señal. Sin resultado anticipado; targets derivados siguen pendientes.</x:v>
+        <x:v>Medir valor incremental del arsenal; experimento aún no ejecutado.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1460,7 +1726,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reda8033ae6c34c3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67905dc0a6fb4b92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Agrega Pitching+/Stuff+ V1, contrafactual de altitud, efecto total y V2 de pesos
- 09: Pitching+/Out+ combinado (5 componentes, z-score, pesos iguales) y escala Stuff+ 100+10z
- 10: contrafactual de altitud (efecto directo, ~0)
- 11: efecto total con transformacion fisica conjunta y bootstrap por pitcher
- 12-14: V2 como sensibilidad (valor por conteo, pesos aprendidos, matriz V1 vs V2 y niveles de evidencia)
- Guia (secciones 26-29), bitacora y README actualizados

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="14" min="1" max="1"/>
@@ -2319,6 +2319,426 @@
       <c r="L32" t="inlineStr">
         <is>
           <t>08_park_holdout.py; 08_park_holdout_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>09_pitching_plus.py</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Pitching+/Out+ combinado y escala Stuff+</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>¿Cómo combinar 5 probabilidades con poblaciones elegibles distintas en un solo score, y mejora el modelo al incluir arsenal+ubicación+altitud+contexto juntos?</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Cada sub-modelo se entrena en su propia población condicional (como en 07/08) pero se anota sobre TODA la población común elegible (arsenal completo + altitud válida) — resuelve que whiff_given_swing/chase/groundball tienen denominadores mutuamente excluyentes por fila. Combinación: z-score de cada probabilidad contra media/SD de train, promedio con pesos iguales (decisión del equipo: pesos de valor de carrera no traducen limpio a estas 5 poblaciones distintas; pesos aprendidos por regresión reabren el problema de PA-terminal que bloqueó xRunValue en 05). Escala final 100+10z.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Sanity check por pitch type reproduce el orden de 03. Arsenal+altitud+contexto mejora cada componente sobre sus versiones puras de 07/08.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>whiff_per_pitch AUC 0.7268 (07, físico puro) -&gt; 0.7531 (full). whiff_given_swing 0.7330 -&gt; 0.7575. groundball 0.6486 -&gt; 0.6531/0.6664. called_strike 0.8790 -&gt; 0.8780/0.8820. chase 0.8419 -&gt; 0.8460/0.8529. Stuff+ (escala 100+10z) por pitch type: Splitter 106-107, Slider 105, Curveball 104, Changeup 103, Cutter 100-101, Sinker 98, Four-Seam 95.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Adoptar el score combinado como Pitching+/Out+ V1 y su escala como Stuff+ V1. Guardar los 5 componentes por separado (09_pitching_plus_scores.csv trae altitude_category y pitcher_anon_id por fila: insumo directo para el contrafactual de altitud siguiente). Pendiente V2: sensibilidad de pesos y pesos aprendidos contra valor de carrera.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>09_pitching_plus.py; 09_pitching_plus_scores.csv; 09_pitching_plus_component_metrics.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>09_pitching_plus.py</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Semantica de componentes y persistencia</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>¿Aplicar cada modelo a toda la poblacion comun mantiene el significado de cada probabilidad?</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Revision metodologica del equipo: chase se aprende solo fuera de zona; aplicarlo a pitches dentro de zona con su ubicacion intacta es extrapolacion. groundball es propension condicionada a contacto.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Correccion: la guia 26.1 llamaba 'contrafactual estandar' a esa aplicacion; solo es valido sin reservas para whiff_given_swing y called_strike.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Columnas renombradas: p_whiff_per_pitch, p_whiff_given_swing, p_groundball_given_contact, p_called_strike, p_chase_given_outside_zone. Nuevo stuff_plus_no_chase (sensibilidad). Modelos y cohorte persistidos en 09_pitching_plus_bundle.pkl (ignorado por git). Resultados de 09 identicos.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Nombres con la poblacion explicita. Reportar siempre stuff_plus_no_chase como sensibilidad.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>09_pitching_plus.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>10_altitude_counterfactual.py</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Contrafactual de altitud (efecto directo)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>¿Cuanto cambia el Stuff+ de un mismo pitch al cambiar solo altitude_category (No vs Extreme, proxy del entorno Harp Helu)?</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>delta_direct = Score(X,Extreme)-Score(X,No) con todo lo demas fijo, usando los modelos exactos de 09. Mas contraste observacional within-pitcher/pitch-type como aproximacion al efecto total. Delta total por modelo (mover IVB/HB/angulos por ambiente) pendiente.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>delta_direct ~ 0 y sin signo estable entre ventanas; el contraste observacional es ruidoso salvo Curveball (negativo en ambas).</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Ventana 2024-25-&gt;2026 (n=87,587): Curveball +0.01, Splitter -0.06, Changeup -0.13, Slider -0.17, Cutter -0.23, Four-Seam -0.30, Sinker -0.34 puntos Stuff+. Ventana 2024-&gt;2025 (n=131,891): Cutter +0.20, Curveball +0.19, Splitter +0.17, Slider +0.17, Changeup +0.11, Four-Seam +0.05, Sinker -0.04. SD dentro de tipo 0.4-0.8. Observado (2026 / 2025): Curveball -0.94 / -1.15, Four-Seam +0.02 / +1.05, Changeup +0.17 / +1.21. Identidad vs 09: max diff 2.8e-14.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>NO reportar aun deltas por pitch shape como hallazgo: el efecto directo es indistinguible de cero. Consistente con 08 (el modelo casi no necesita saber la altitud) y con la hipotesis de que el efecto viaja via movimiento observado. Siguiente: delta total con features desplazadas por deltas within-pitcher empiricos + bootstrap por pitcher. Ojo: el promedio de 5 z-scores diluye el efecto (solo la parte whiff es sensible), orden de magnitud ~1 punto.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>10_altitude_counterfactual.py; 10_altitude_delta_by_*.csv; 10_altitude_observed_contrast.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>11_altitude_total_effect.py</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Delta total de altitud + bootstrap por pitcher</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>¿Cuanto cambia el Stuff+ de un pitch por pitch type/shape al transportarlo a Extreme Altitude (proxy Harp Helu) con su fisica cambiando como historicamente cambia ese tipo?</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Transformacion conjunta por tipo (celdas pitcher x tipo x anio, solo historial, validada en la temporada futura) que desplaza solo IVB, HB, VertApprAngle, HorzApprAngle (+ diffs vs FB); release como placebo; cohorte No observado -&gt; Extreme; chequeo inverso; bootstrap por pitcher B=500 (celdas y cohorte); regla IC95% y umbral de relevancia 1 pt.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Efectos por tipo &lt; 1 punto Stuff+. Signo de rectas/Changeup depende de los pesos iguales (groundball); solo Curveball y Slider robustos a quitarlo.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2024-25-&gt;2026: Curveball -0.78 [-0.99,-0.58], Slider -0.33 [-0.42,-0.24], Four-Seam +0.28 [+0.12,+0.45] (sin groundball -1.97), Sinker +0.36 (sin GB -0.35), Changeup +0.28 (sin GB -0.19), Cutter +0.63 (sin GB -0.05 incierto), Splitter -0.83 [-1.56,+0.80] incierto (8 celdas). Four-Seam contribuciones: whiff -1.05/-0.59, GB +2.25. Validacion transformacion Four-Seam IVB -3.82 vs -3.90 observado. Chequeo inverso mismo signo en 7 tipos.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No titular ganancia/perdida en rectas hasta tener pesos de valor de carrera (V2); reportar componentes. Curveball y Slider: perdida pequena y robusta. Splitter/Cutter: baja confianza (pocas celdas). Efecto viene de la fisica desplazada, no de la etiqueta (apoya 08 y H1/H4).</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>11_altitude_total_effect.py; 11_altitude_total_*.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>12_weight_sensitivity.py</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>V2 paso 1: sensibilidad al peso de groundball</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>¿En que peso relativo de groundball cambia el signo del delta total por pitch type?</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Curva delta(w) exacta (score lineal en z) y punto de quiebre con IC95% bootstrap por pitcher, sin tocar V1.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Rectas y Changeup positivas en V1 solo por poco.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Quiebre Four-Seam 0.88 [0.80,0.95] (2026) y 0.76 (2025); Sinker 0.49; Changeup 0.40; Curveball negativo con cualquier w&gt;=0.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>La conclusion sobre rectas depende de una razon groundball/whiff que V1 fija en 1 sin respaldo.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>12_gb_weight_breakeven.csv; 12_gb_weight_curve.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>13_count_value_weights.py</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>V2 pasos 2-5: valor por conteo y pesos</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>¿Que pesos del compuesto se ligan a valor de carrera observable, y son estables entre ventanas?</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Cadena de Markov por conteo (12 estados), transiciones empiricas de PitchCall, pagos terminales de The Book/FanGraphs 2006 (excepcion autorizada solo para eventos terminales; guia 29.1). Regresion no negativa con ridge leve sobre los 5 z, bootstrap por pitcher. RunsScored descartado (sencillo 0.25 vs out 0.02).</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Groundball pesa ~0 a nivel pitch; estabilidad estricta NO cumplida (IC no solapan en 2 de 5; dif. max .061).</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Pesos V2 (2025/2026): called_strike .370/.416, chase .305/.282, whiff_per_pitch .264/.303, whiff_given_swing .061/.000, groundball .000/.000 (IC hasta .026). Fuera de muestra hacia adelante: RMSE nulo .21925, V1 .21840 (-0.78% MSE), V2 .21702 (-2.02%), V2 vs V1 -1.25% [1.11,1.40].</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Leer groundball como 'pequeno', no cero (solo 18% BIP, modelo AUC .65, indice lineal no captura P(contacto)xp_GB; SI paga +.12 runs mas que un elevado por BIP). V2 se reporta como sensibilidad; V1 permanece.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>13_count_value_weights.py; 13_*.csv; 13_v2_bundle.pkl</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>14_v1_v2_altitude_matrix.py</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>V2 paso 6: matriz V1 vs V2 y niveles de evidencia</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>¿Cambia la conclusion ambiental por pitch type al usar pesos ligados a valor de carrera?</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Recombinacion de replicas bootstrap de 11 con V1, V2 propio, V2 cruzado y V2-stuff; niveles Robusto/Condicional/Incierto con criterios explicitos.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>V1-&gt;V2 (2026): Four-Seam +0.28 -&gt; -1.44, Sinker +0.36 -&gt; -0.47, Changeup +0.28 -&gt; -0.12 (Condicional); Slider -0.33/-0.43 y Curveball -0.78/-0.22 (Robusto, &lt;1 pt); Cutter y Splitter Incierto (&lt;30 celdas).</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Four-Seam pierde por whiff (-1.13 pts), consistente con H1; V2-stuff -2.2. Curveball en V2 viene de called strike (ubicacion fija: lectura cautelosa).</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Decision pendiente: escala oficial (recomendado V1 oficial + V2 como lectura ligada a valor).</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>14_v1_v2_altitude_matrix.py; 14_evidence_levels.csv</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="14" min="1" max="1"/>
@@ -2608,7 +3028,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>altitude_counterfactual.py (número pendiente de asignar al crearse)</t>
+          <t>10_altitude_counterfactual.py</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -2618,12 +3038,12 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado (V1: efecto directo)</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>DeltaScore por pitch type/shape/pitcher.</t>
+          <t>Delta directo ~0 y inestable entre ventanas (Bitácora ID 34). Falta delta total (movimiento por ambiente) para el entregable de altitud.</t>
         </is>
       </c>
     </row>
@@ -2638,7 +3058,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>altitude_uncertainty.py (número pendiente de asignar al crearse)</t>
+          <t>(cubierto por 11_altitude_total_effect.py)</t>
         </is>
       </c>
       <c r="D10" s="12" t="inlineStr">
@@ -2648,12 +3068,12 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado (V1, bootstrap por pitcher en 11)</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Resultados con incertidumbre.</t>
+          <t>Bootstrap por pitcher B=500 con IC95% para delta total por tipo y shape.</t>
         </is>
       </c>
     </row>
@@ -2774,6 +3194,126 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>AUC casi identico al pitcher holdout de 07 en los 5 targets (deltas entre -0.0083 y +0.0003). Robustez ambiental confirmada para el boosting V1. Ver Bitácora ID 31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pitching+/Out+ combinado y escala Stuff+</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>09_pitching_plus.py</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Combinar los 5 sub-modelos (stuff+ubicacion+arsenal+altitud+contexto) en un score unico y normalizarlo a escala Stuff+ (100+10z).</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Cerrado (V1, pesos iguales)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Stuff+ V1 por pitch, con los 5 componentes guardados por separado. Sanity check por pitch type coherente con 03. Arsenal+altitud+contexto mejora cada componente vs 07/08. Ver Bitácora ID 32. Pendiente: pesos aprendidos contra valor de carrera (V2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Delta total por ambiente</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_altitude_total_effect.py</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Score(X^Extreme,Extreme)-Score(X^No,No): desplazar features fisicas (IVB, HB, angulos de aproximacion, etc.) por deltas within-pitcher/type/year empiricos, de forma consistente.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Cerrado (V1)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Efectos &lt; 1 pt; signo de rectas depende de pesos iguales (Bitácora ID 35). Falta V2 con pesos de valor de carrera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Pesos de valor de carrera (V2)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>12_, 13_ y 14_ (sensibilidad, pesos, matriz)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Reemplazar pesos iguales por pesos ligados a valor de carrera / run expectancy por conteo y medir sensibilidad; decide el neto de las rectas en altitud.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Cerrado (sensibilidad; V1 permanece)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Rectas y Changeup cambian de signo con V2; Curveball y Slider robustos (&lt;1 pt). Estabilidad estricta de pesos no cumplida. Ver Bitácora ID 36-38 y guia 29. Decision pendiente: escala oficial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Perfil ideal y recomendaciones operativas</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>(número pendiente de asignar al crearse)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Traducir la tabla de niveles de evidencia (robusto/condicional/incierto) a perfil fisico ideal y recomendaciones de scouting.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Planeado</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Entregables 2 y 3.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correcion a los modelos
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="14" min="1" max="1"/>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Adoptar HistGradientBoostingClassifier como modelo principal V1 mientras no se resuelva libomp. called_strike/chase son el primer Location+ real del proyecto. Arsenal excluido aquí a propósito (100% NaN en test bajo pitcher holdout); su combinación con boosting queda para Pitching+.</t>
+          <t>Adoptar HistGradientBoostingClassifier como modelo principal V1 mientras no se resuelva libomp. called_strike/chase son el primer Location+ real del proyecto. Arsenal excluido aquí a propósito (100% NaN en test bajo pitcher holdout); su combinación con boosting queda para Pitching+. [Nota 25/09/2026: la familia 'stuff' incluia angulos que reconstruyen la ubicacion (R2 0.995); su AUC no es Stuff+ fisico. Ver ID 41 y guia 32]</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>El modelo generaliza bien a un entorno no visto sin necesitar saber en cuál está. Hipótesis de por qué: las features usadas (IVB, HB, etc.) son movimiento OBSERVADO, no spin teórico, así que ya incorporan el efecto físico de la altitud en cada pitch medido; el modelo aprende la relación movimiento-&gt;outcome, que parece estable entre entornos. Esto es evidencia adicional a favor de H4 (shape over label). No implica ausencia de efecto de altitud: la EDA ya mostró que la distribución de IVB/HB sí cambia con altitud; lo que se sostiene es la relación aprendida entre esas features y el outcome.</t>
+          <t>El modelo generaliza bien a un entorno no visto sin necesitar saber en cuál está. Hipótesis de por qué: las features usadas (IVB, HB, etc.) son movimiento OBSERVADO, no spin teórico, así que ya incorporan el efecto físico de la altitud en cada pitch medido; el modelo aprende la relación movimiento-&gt;outcome, que parece estable entre entornos. Esto es evidencia adicional a favor de H4 (shape over label). No implica ausencia de efecto de altitud: la EDA ya mostró que la distribución de IVB/HB sí cambia con altitud; lo que se sostiene es la relación aprendida entre esas features y el outcome. [Nota 25/09/2026: la interpretacion H4 se apoya en features que codifican ubicacion; rehacer con 16. Ver ID 41]</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Adoptar el score combinado como Pitching+/Out+ V1 y su escala como Stuff+ V1. Guardar los 5 componentes por separado (09_pitching_plus_scores.csv trae altitude_category y pitcher_anon_id por fila: insumo directo para el contrafactual de altitud siguiente). Pendiente V2: sensibilidad de pesos y pesos aprendidos contra valor de carrera.</t>
+          <t>Adoptar el score combinado como Pitching+/Out+ V1 y su escala como Stuff+ V1. Guardar los 5 componentes por separado (09_pitching_plus_scores.csv trae altitude_category y pitcher_anon_id por fila: insumo directo para el contrafactual de altitud siguiente). Pendiente V2: sensibilidad de pesos y pesos aprendidos contra valor de carrera. [Nota 25/09/2026: score de 09 = Pitching+, no Stuff+; la mejora vs 07 no se atribuye a arsenal/altitud (ablacion: arsenal -0.0026 AUC whiff, altitud ~0). Ver ID 41]</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2859,6 +2859,486 @@
       <c r="L41" t="inlineStr">
         <is>
           <t>15_*.csv; guia seccion 31</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>16_three_scores.py</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>Correccion post-auditoria (Bloque A)</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>Separar Stuff+ fisico sin fuga de ubicacion, Location+ y Pitching+; cobertura para pitchers nuevos; pesos sin pesos iguales arbitrarios.</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>Stuff+ sin angulos de release/aproximacion; tres familias x 5 componentes; variantes base/arsenal; pesos no negativos contra valor por conteo con OOF del historial; V1 como sensibilidad.</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>Fuga de ubicacion eliminada (R2 0.995 -&gt; 0.15/0.10). Stuff+ fisico AUC whiff ~0.63 (nuevos ~0.62). Los tres scores superan al nulo por conteo; pesos aprendidos &gt; V1 en las 3 familias. Cobertura 100%.</t>
+        </is>
+      </c>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>Red. MSE vs nulo 2026: Pitching+ 2.10%, Location+ 1.93%, Stuff+ 0.10% (IC excluye 0). V1: 0.85/0.73/0.05%. Corr Location+/Pitching+ 0.957. Calibracion: GB subestimado hasta 7 pp (deriva de temporada).</t>
+        </is>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
+        <is>
+          <t>Adoptar los tres scores de 16. Pesos aprendidos OOF como oficiales (reemplaza V1 oficial de ID 40; reversible). 07-15 pasan a arquitectura experimental. Siguen Bloques B, C y D.</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L42" s="1" t="inlineStr">
+        <is>
+          <t>16_three_scores.py; 16_*.csv; guia seccion 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>17_sequence_and_contact.py</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>Secuencia, PA, contacto y RE LMB</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>¿Se puede ordenar pitches y reconstruir PA? ¿Hay evidencia de H3 en LMB?</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr">
+        <is>
+          <t>Orden por timestamp UUID v1; PA por cambio de bateador o pitch terminal; hard-hit &gt;=95 y weak &lt;60 (Statcast); HR|BIP; RE por conteo x outs; H3 por altitud y within-pitcher.</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
+        <is>
+          <t>PA validas: 98.8% empiezan en 0-0, 99.0% terminan en terminal, 99.7% de conteos coherentes. H3 soportada: ventaja GB-FB +0.14 (No) vs +0.25 runs (Extreme).</t>
+        </is>
+      </c>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>Within-pitcher Extreme-No: HR/FB +4.7 pp [2.0, 7.7], hard-hit +2.7 pp, GB +5.1 pp. Carreras/juego: No 9.05, Extreme 13.66.</t>
+        </is>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>Adoptar la secuencia y el RE LMB (reemplaza The Book). Barrel no se implementa (no replicable).</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K43" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L43" s="1" t="inlineStr">
+        <is>
+          <t>17_*.csv; 17_pitch_sequence.parquet; guia 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>18_three_scores_v2.py</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>Tres scores V2 (9 componentes) y pesos de Stuff+</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>¿Los scores con targets completos y valor LMB validan? ¿Como ponderar Stuff+?</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr">
+        <is>
+          <t>9 componentes; Pitching+ con Outs/Inning/prev_pitch_type; pesos OOF contra RE LMB; Stuff+ con pesos de evento de Pitching+ sin called strike; chequeo a nivel pitcher.</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>Pesos propios de Stuff+ mal identificados (called strike 0.60, orden implausible, corr pitcher 0.017). Con la regla nueva: Splitter 112, Slider 106, Changeup 105 ... Sinker 93. Componentes de contacto con peso ~0.</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>Red. MSE 2026: Pitching+ 1.80%, Location+ 1.70%, Stuff+ ~0. Pitcher: Stuff+ corr 0.152 [0.043, 0.272], split-half 0.989; valor realizado 0.221, split-half 0.341.</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>18 = scores oficiales. Pendiente: termino estructural de valor en contacto (H3 en el score), recalibracion por temporada y validacion formal (Bloque C).</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t>18_*.csv; guia 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>18_three_scores_v2.py</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>Rama de contacto y ablacion (ultima modificacion de arquitectura)</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>¿Monetizar explicitamente el contacto (P(BIP) x E[valor | BIP]) mejora el valor fuera de muestra y da efectos ambientales coherentes?</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>Componente contact_value; Stuff+/Location+ con RE general (neutrales), Pitching+ con RE por entorno + altitude_category; ablacion A' (sin rama) vs B en la misma corrida; contrafactual No -&gt; Extreme.</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>B empeora el valor fuera de muestra en ambas ventanas y a nivel pitcher. La coherencia ambiental es correcta en signo (mas dano en Extreme, menos en pitches de roletazo) pero pequena.</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>Pitching+ 2026: A' 1.66% vs B 1.56%. Pitcher: A' 0.193 vs B 0.093 (Stuff+ 0.153 vs 0.098). Delta contact_value Extreme-No: -0.21 a -0.35 runs/100; GB alto -0.20 vs bajo -0.30.</t>
+        </is>
+      </c>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>Rama como modulo explicativo de H3, no en el score. Oficial = A'. Arquitectura congelada; siguiente: Bloque C.</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>18_*.csv; 18_contact_env_coherence.csv; guia 34</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>19_validation.py</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>Bloque C: validacion formal</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>¿La arquitectura congelada generaliza a pitchers no vistos, temporadas futuras y entornos no vistos? ¿Esta calibrada? ¿Que tan estable es Stuff+?</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>GroupKFold 5 por pitcher; season-forward de 18; park holdout en 3 direcciones; split-half, año a año y prediccion t -&gt; t+1 con IC; calibracion (Brier, pendiente, deciles) y recalibracion 2025 -&gt; 2026.</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>Stuff+ muy estable (split-half 0.99, año a año 0.77-0.78; valor observado 0.22-0.26) y generaliza (AUC igual en Extreme no visto). Location+/Pitching+ ~1.7% de reduccion de MSE en CV. La recalibracion no ayuda (deriva de temporada). Ningun score supera al valor observado en correlacion t+1.</t>
+        </is>
+      </c>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>CV red. MSE: Pitching+ 1.66% ± 0.12, Location+ 1.74% ± 0.11, Stuff+ 0.01%. Park -&gt; Extreme AUC whiff Pitching+ 0.7504 (CV mismas filas 0.7502). Corr t+1: Stuff+ 0.20/0.17, observado 0.22/0.26, combinado 0.25/0.27.</t>
+        </is>
+      </c>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>Bloque C cerrado sin descongelar. Fallos conocidos documentados (guia 35.4). Siguiente: Bloque D.</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K46" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>19_*.csv; 19_cv_oof.parquet; guia 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>20_altitude_physics.py</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>D1-D2: forma de la transformacion y gradiente</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>¿Aditiva o multiplicativa? ¿Medium cae entre No y Extreme?</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr">
+        <is>
+          <t>Cuatro formas contra 'sin cambio', aprendidas con historial y evaluadas en celdas de la temporada futura; regla de desempate fijada antes. Gradiente within-pitcher con bootstrap.</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
+        <is>
+          <t>Multiplicativas &gt;&gt; aditiva (RMSE 1.15 contra 1.53 in). Elegida mult_global_var: IVB x0.77, HB x0.71 en Extreme. Medium entre No y Extreme en los 7 tipos.</t>
+        </is>
+      </c>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>r Magnus: Medium 0.814, Extreme 0.743. RMSE promedio: mult_tipo 1.150, mult_global_var 1.155, magnus 1.192, aditiva 1.525, sin cambio 3.368.</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>Adoptar la transformacion multiplicativa global por variable (2 parametros).</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L47" s="1" t="inlineStr">
+        <is>
+          <t>20_*.csv; guia 36.1-36.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>21_altitude_stuff_delta.py</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>D3-D4: delta Stuff+ limpio y H1-H4</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>¿Cuanto cuesta en Stuff+ el cambio fisico de altitud? ¿Lo confirma lo observado?</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>Delta modelado (transformacion de 20) con bootstrap por pitcher, chequeo inverso, sensibilidad a la forma y contraste observado del Stuff+ del mismo pitcher; pruebas de H2 y H4.</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>Four-Seam -4.8 y Sinker -2.8 confirmados por lo observado (-4.7 y -1.6). Slider/changeup/curva: perdida modelada de 1.2-2.3 que no aparece en el neto observado.</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>Niveles: Robusto FF y SI; Condicional CH, SL y CU; Incierto FC y FS. H2: CH/FS pierden 0.76 [0.46, 1.16] menos que los Magnus. H4: mismas rpm dan 76% del movimiento en Extreme.</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>Regla de Robusto endurecida: exige confirmacion observada. Reemplaza las secciones 28-30.</t>
+        </is>
+      </c>
+      <c r="J48" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L48" s="1" t="inlineStr">
+        <is>
+          <t>21_*.csv; guia 36.3-36.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>22_profile_recommendations_export.py</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>D5-D7: perfil, recomendaciones, proyeccion y congelamiento</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>¿Que perfil fisico funciona en altitud? ¿Como se usa para scouting? ¿Que se entrega al dashboard?</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>Lifts del quintil superior de Stuff+ en Extreme (2025 -&gt; 2026), resiliencia, estabilidad por tipo, validacion contra whiff/chase reales; proyeccion por pitcher; manifiesto y simulate_pitch.</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
+        <is>
+          <t>El Stuff+ alto en Extreme se traduce en mas whiff y chase reales (6 de 7 tipos, IC &gt; 0). Perfil casi todo compartido con nivel del mar. Rectas de mucho ride pierden mas. Correlacion de rangos mar vs Harp Helu 0.961.</t>
+        </is>
+      </c>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>Proyeccion 2026: 369 pitchers, delta medio -2.95 (rango -8.3 a 0). simulate_pitch verificado exactamente contra la proyeccion.</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>Invalida el perfil de 15. Outputs congelados; siguiente: producto (dashboard, documento, pitch).</t>
+        </is>
+      </c>
+      <c r="J49" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L49" s="1" t="inlineStr">
+        <is>
+          <t>22_*.csv; 22_dashboard_manifest.json; guia 36.5-36.7</t>
         </is>
       </c>
     </row>
@@ -2884,7 +3364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="14" min="1" max="1"/>
@@ -3223,7 +3703,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Stuff+/Location+/Pitching+ reportables.</t>
+          <t>Stuff+/Location+/Pitching+ reportables. Insumos congelados en 22_dashboard_manifest.json (guia 36.7).</t>
         </is>
       </c>
     </row>
@@ -3253,7 +3733,7 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Entregable final.</t>
+          <t>Entregable final. Insumos congelados en 22_dashboard_manifest.json (guia 36.7).</t>
         </is>
       </c>
     </row>
@@ -3434,6 +3914,166 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Ver Bitácora ID 40 y guia 31. Pendiente: dashboard y documento tecnico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>9.8</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>Correccion post-auditoria (Bloque A)</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>16_three_scores.py</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Stuff+ fisico sin fuga de ubicacion, Location+ y Pitching+ separados, cobertura total y pesos aprendidos OOF.</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>Tres scores 100+10z por pitch; base para B, C y D. Ver Bitacora ID 41 y guia 32.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>9.9</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Bloque B: secuencia, outs y contacto</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>17_sequence_and_contact.py; 18_three_scores_v2.py</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Orden por UUID, prev_pitch_type, out_within_PA, hard-hit/HR|contacto, valor por conteo x outs.</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>Secuencia, PA, prev_pitch_type, out_within_PA, hard-hit/HR, RE LMB; scores oficiales en 18. Ver Bitacora ID 42-43 y guia 33.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>9.95</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>Bloque C: suite de validacion</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>19_validation.py</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>GroupKFold de pitcher, season-forward, park holdout, reliability y estabilidad por pitcher sobre 16.</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>Tabla de salida y fallos conocidos (guia 35); arquitectura sigue congelada. Bitacora ID 45.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>9.97</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Bloque D: altitud sobre scores limpios</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>20_altitude_physics.py; 21_altitude_stuff_delta.py; 22_profile_recommendations_export.py</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Transformacion aditiva vs multiplicativa, gradiente Medium, deltas por shape y perfil/recomendaciones.</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>Transformacion multiplicativa validada, delta Stuff+ con confirmacion observada, H1-H4, perfil y recomendaciones; outputs congelados. Bitacora ID 46-48.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>9.93</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>Rama de contacto y congelamiento de arquitectura</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>18_three_scores_v2.py</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Ablacion A' vs B de P(BIP) x E[valor | BIP]; decidir score oficial y congelar.</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Oficial A' (sin rama); rama como modulo explicativo de H3. Bitacora ID 44, guia 34.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dashboard Pitching Decision System (fases 1-4) y capa de datos
- 23_dashboard_data.py: tablas del dashboard y reglas de producto.
- dashboard/: app Streamlit con Roster, Player, Simulator, Scouting y Game;
  motor (engine.py) verificado contra los scores oficiales de 18.
- Analisis de factibilidad del diseño, wireframes, requirements.txt.
- Guia (seccion 37), bitacora (ID 49-52) y README actualizados.
- .gitignore: se quita la regla '.json' (no ignoraba nada util) y se
  excluyen .claude/, dashboard/data/ y dashboard/state/.

Punto de control previo a las correcciones de la auditoria 2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="14" min="1" max="1"/>
@@ -3339,6 +3339,246 @@
       <c r="L49" s="1" t="inlineStr">
         <is>
           <t>22_*.csv; 22_dashboard_manifest.json; guia 36.5-36.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>23_dashboard_data.py; dashboard/</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard fase 1 (Roster + Player)</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>¿Que del diseño (design thinking + wireframes) sostienen los modelos? ¿Como se integra?</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr">
+        <is>
+          <t>Analisis de factibilidad por pantalla; reconstruccion de equipos por co-aparicion; rol inferido; fechas desde UUID; capa de datos con reglas explicitas; app Streamlit con el sistema visual del wireframe.</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>Roster y Player Overview funcionando con datos reales. 19 equipos reconstruidos, 4-5 locales en Extreme. Semaforo relativo (el absoluto marcaba al 52%).</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>2026: alertas 25% red / 29% yellow / 46% green; inbox 97 atencion + 108 review + 85 oportunidades; 538 pitchers con tendencia semanal.</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>Roster configurable (dataset anonimo). Recomendaciones sin prescripcion de uso. Siguiente: Simulator.</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L50" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard_Analisis_Factibilidad.md; 23_dashboard_data.py; dashboard/; guia 37</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>dashboard/lib/engine.py; dashboard/views/simulator.py</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard fase 2: Simulator</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>¿Como simular el mismo pitch a nivel del mar vs Harp Helu y escenarios what-if sin romper la consistencia con los scores oficiales?</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>Motor que reutiliza los modelos de 18; what-if poblacional (desplaza los pitches reales); prospectos = dispersion de la liga recentrada; Location+ en rejilla; experimentos persistidos.</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
+        <is>
+          <t>El motor reproduce exactamente los scores de 18 y la proyeccion de 22. Calificar el 'pitch promedio' era inconsistente por la no linealidad (100 vs 107).</t>
+        </is>
+      </c>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>Diff max 1.4e-14; Four-Seam 00776: 107.02 -&gt; 100.23 (identico a Player); +2 in de IVB: Harp 100.2 -&gt; 103.5.</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>Simulator listo. Siguiente: Scouting.</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="inlineStr">
+        <is>
+          <t>dashboard/; guia 37.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>dashboard/views/scouting.py; dashboard/lib/engine.py</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard fase 3: Scouting + hallazgo de variante</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>¿Como apoyar seleccion (perfil, candidatos, prospectos, comparacion, shortlist) sin sesgos de comparacion?</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>Perfil ideal por tipo; explorador con señales Stuff+ vs resultados; prospectos por dispersion recentrada; comparador; shortlist persistida; referencia de la liga con la misma variante del modelo.</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>Slider/changeup: el delta de altitud depende de la variante (con arsenal -2.3/-2.9; sin arsenal -0.2/-0.8), y la variante fisica coincide con lo observado. Sin referencia de la misma variante los prospectos salian inflados.</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>Corr Stuff+ Harp vs valor/100 = 0.25 (n &gt;= 300). Referencia base: 887 pitcher x tipo, 369 pitchers, 1.4 s.</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>Scouting listo. El hallazgo matiza la lectura 'Condicional' de la guia 36. Siguiente: Game.</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>guia 37.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>dashboard/views/game.py; dashboard/lib/engine.py</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard fase 4: Game</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>¿Como dar una lectura tactica rapida y honesta (sin 'mejor pitch') que refleje la altitud?</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>Tarjetas por pitch con calidad esperada en su mejor zona; heatmaps de Pitching+ y del costo del contacto en el count (rama de contacto, RE del entorno); lectura en una linea; Why? bajo demanda.</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>Lecturas coherentes con el beisbol (0-2: four-seam arriba). El costo del contacto se mide contra el valor del count: ~0 en counts neutros y mayor con dos strikes, donde la altitud lo encarece.</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>00776 Four-Seam 0-2 vs derecho: costo en zona 4.0 (Harp) vs 2.4 (mar) runs/100; rejilla ~0.25 s.</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard completo (5 pantallas). Siguiente: documento tecnico y pitch.</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>guia 37.7</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3958,7 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>23_dashboard_data.py; dashboard/</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
@@ -3728,12 +3968,12 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado (5 pantallas)</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Entregable final. Insumos congelados en 22_dashboard_manifest.json (guia 36.7).</t>
+          <t>Roster, Player, Simulator, Scouting y Game con datos reales; motor verificado contra 18. Bitacora ID 49-52, guia 37.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auditoria 2: titular de altitud fisico, Fit = calidad proyectada, alertas por exceso
- 21: variantes fisica (titular) y oficial (sensibilidad); niveles de evidencia por variante
- 22: nivel Harp = Stuff+ oficial a nivel del mar + delta fisico; textos de recomendacion
- 23: Fit = percentil del Stuff+ proyectado; alerta = pierde mas de lo esperado para su nivel y tipo
- Dashboard: motor hibrido (population_table, prospect), Simulator sin crash 2025, Roster/Player/Scouting con la nueva semantica
- Guia 38, bitacora 53-54, README

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="14" min="1" max="1"/>
@@ -3579,6 +3579,130 @@
       <c r="L53" s="1" t="inlineStr">
         <is>
           <t>guia 37.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>21_altitude_stuff_delta.py; 22_profile_recommendations_export.py</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria 2: titular de altitud por variante</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>¿Que variante del modelo debe dar el efecto de altitud titular?</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>Variante fisica (sin arsenal para todos) vs oficial (con arsenal)</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>La fisica coincide con lo observado del mismo pitcher; la oficial exagera slider/changeup por la separacion contra la recta</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>2026 fisica vs obs: FF -5.43/-5.41, SI -2.87/-2.47, CU -1.25/-1.06, CH -0.60/-0.91, SL -0.16/+0.27</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>Titular = fisica; oficial = sensibilidad. Nivel Harp = oficial mar + delta fisico</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="inlineStr">
+        <is>
+          <t>guia 38.1; 21_evidence_levels*.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>23_dashboard_data.py; dashboard/</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria 2: Fit y alertas</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>¿El Fit y las alertas premian a pitchers mediocres?</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr">
+        <is>
+          <t>Fit = percentil de delta vs Fit = Stuff+ proyectado; alerta = residuo del delta dado Stuff+ y tipo</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>Los mejores pitchers pierden mas puntos (Spearman -0.43); la nueva alerta es independiente del nivel (Spearman 0.03)</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>Stuff+ por Fit: Strong 106.9 / Poor 96.3; alertas 39 rojas, 65 amarillas, 267 verdes (n = 371)</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>Fit = calidad proyectada en Harp; alerta = pierde mas de lo esperado. Pantallas actualizadas; bug del Simulator corregido</t>
+        </is>
+      </c>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>guia 38.2-38.4</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="14" min="1" max="1"/>
@@ -4317,6 +4441,38 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>9.98</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>Auditoria 2: Fit, alertas y titular de altitud</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>21, 22, 23; dashboard/</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>Corregir definiciones antes del documento tecnico</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>Titular fisico y Fit/alertas independientes del nivel; listo para documento tecnico</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="E2:E50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
Tasa de roletazos solo con bolas en juego y cierre de pendientes de la bitacora
- 23: gb_rate filtra is_ball_in_play == 1 (correccion de Dani). Antes contaba 74,638 filas que no son bolas en juego (72,818 fouls); ahora coincide con la definicion de la guia 22 (liga 45.84%, 107,118 BIP).
- Sinker >= 30% del arsenal: 51.9% vs 46.2% (2025) y 51.2% vs 46.4% (2026); antes 41% vs 35-36%. La brecha casi no cambia; por cuartil de rectas la tasa queda plana.
- 24 y Scouting > Arsenal ideal: definicion documentada en docstring y en pantalla. Pendientes del valor realizado y Spearman de composiciones sin cambio.
- README (A7), guia 42.5 corregida y nueva 42.10 (incluye la cifra corregida del What-if del 00776: 102.3 en Harp Helu, no 100.7).
- Bitacora: fila 71; filas 14, 15, 16, 21, 28 y 49 y roadmap 6 y 10 cerradas con nota de donde quedaron; rangos de las tablas de Excel al dia.
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -153,7 +153,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BitacoraTable" displayName="BitacoraTable" ref="A1:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BitacoraTable" displayName="BitacoraTable" ref="A1:L72" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="12">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Fecha"/>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoadmapTable" displayName="RoadmapTable" ref="A1:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RoadmapTable" displayName="RoadmapTable" ref="A1:F25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="6">
     <tableColumn id="1" name="Orden"/>
     <tableColumn id="2" name="Etapa"/>
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="14" min="1" max="1"/>
@@ -1283,12 +1283,12 @@
       </c>
       <c r="I15" s="12" t="inlineStr">
         <is>
-          <t>Implementar A/B y reportar efecto incremental.</t>
+          <t>Implementar A/B y reportar efecto incremental. Actualizacion 14/10/2026: no implementado como script; la decision por capa quedo fijada en 16/18 (guia 32.2); fuera de alcance para la entrega.</t>
         </is>
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
@@ -1343,12 +1343,12 @@
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Implementar sobre el modelo que incluya ambiente y agregar por pitch type/shape/pitcher.</t>
+          <t>Implementar sobre el modelo que incluya ambiente y agregar por pitch type/shape/pitcher. Actualizacion 14/10/2026: se hizo con otros numeros: contrafactual de altitud en 10_altitude_counterfactual.py (ID 34) y efecto total en 11_altitude_total_effect.py (ID 35); version vigente sobre Stuff+ limpio en 21_altitude_stuff_delta.py (ID 47, guia 36).</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">
@@ -1403,12 +1403,12 @@
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>Reportar intervalos de incertidumbre junto a deltas.</t>
+          <t>Reportar intervalos de incertidumbre junto a deltas. Actualizacion 14/10/2026: se hizo con otros numeros: bootstrap por pitcher en 11_altitude_total_effect.py (ID 35); version vigente sobre Stuff+ limpio en 21_altitude_stuff_delta.py (ID 47, guia 36).</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
@@ -1703,12 +1703,12 @@
       </c>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>Experimento pendiente. Actualización 24/09/2026: primero revisar 05_target_definitions.py; no entrenar aún.</t>
+          <t>Experimento pendiente. Actualización 24/09/2026: primero revisar 05_target_definitions.py; no entrenar aún. Actualizacion 14/10/2026: realizado en 06_arsenal_incremental_value.py (ID 29).</t>
         </is>
       </c>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K22" s="12" t="inlineStr">
@@ -2123,12 +2123,12 @@
       </c>
       <c r="I29" s="12" t="inlineStr">
         <is>
-          <t>Retomar experimento pospuesto, ahora numerado 06. No anticipar mejora.</t>
+          <t>Retomar experimento pospuesto, ahora numerado 06. No anticipar mejora. Actualizacion 14/10/2026: realizado en 06_arsenal_incremental_value.py (ID 29).</t>
         </is>
       </c>
       <c r="J29" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K29" s="12" t="inlineStr">
@@ -3383,12 +3383,12 @@
       </c>
       <c r="I50" s="1" t="inlineStr">
         <is>
-          <t>Roster configurable (dataset anonimo). Recomendaciones sin prescripcion de uso. Siguiente: Simulator.</t>
+          <t>Roster configurable (dataset anonimo). Recomendaciones sin prescripcion de uso. Siguiente: Simulator. Actualizacion 14/10/2026: dashboard completo (5 pantallas); ver IDs 50-52 y 60-70.</t>
         </is>
       </c>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>En curso</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -4695,6 +4695,68 @@
       <c r="L71" s="1" t="inlineStr">
         <is>
           <t>guia 42.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B72" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C72" s="1" t="inlineStr">
+        <is>
+          <t>23_dashboard_data.py; 24_arsenal_harp.py; views/scouting.py</t>
+        </is>
+      </c>
+      <c r="D72" s="1" t="inlineStr">
+        <is>
+          <t>Tasa de roletazos solo con bolas en juego</t>
+        </is>
+      </c>
+      <c r="E72" s="1" t="inlineStr">
+        <is>
+          <t>¿La tasa de roletazos de Arsenal ideal usa la definicion de la seccion 22?</t>
+        </is>
+      </c>
+      <c r="F72" s="1" t="inlineStr">
+        <is>
+          <t>Filas con hit_type conocido (incluye fouls) vs solo is_ball_in_play == 1</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="inlineStr">
+        <is>
+          <t>Contaba 74,638 filas que no son bolas en juego (72,818 fouls). Con BIP: sinker &gt;= 30% 51.9% vs 46.2% (2025) y 51.2% vs 46.4% (2026); por cuartil de rectas la tasa queda plana</t>
+        </is>
+      </c>
+      <c r="H72" s="1" t="inlineStr">
+        <is>
+          <t>Liga 45.84% (107,118 BIP, igual a la seccion 22); brecha +5.7 / +4.8 pp, IC sin traslape</t>
+        </is>
+      </c>
+      <c r="I72" s="1" t="inlineStr">
+        <is>
+          <t>gb_rate solo con bolas en juego; pendientes y Spearman de 24 sin cambio</t>
+        </is>
+      </c>
+      <c r="J72" s="1" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="L72" s="1" t="inlineStr">
+        <is>
+          <t>guia 42.5, 42.10; 24_arsenal_contraste.csv</t>
         </is>
       </c>
     </row>
@@ -4934,12 +4996,12 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado (fuera de alcance)</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Decisiones sustentadas por evidencia. Sin número fijo todavía: se asigna al crearse, siguiendo el correlativo real en disco (evita colisiones como las de 06/07/08, ver Bitácora ID 21, 28, 30, 31).</t>
+          <t>Decisiones sustentadas por evidencia. Sin número fijo todavía: se asigna al crearse, siguiendo el correlativo real en disco (evita colisiones como las de 06/07/08, ver Bitácora ID 21, 28, 30, 31). Actualizacion 14/10/2026: Decision por capa fijada en 16/18; no se implemento como script.</t>
         </is>
       </c>
     </row>
@@ -5054,12 +5116,12 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Planeado</t>
+          <t>Cerrado</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Stuff+/Location+/Pitching+ reportables. Insumos congelados en 22_dashboard_manifest.json (guia 36.7).</t>
+          <t>Stuff+/Location+/Pitching+ reportables. Insumos congelados en 22_dashboard_manifest.json (guia 36.7). Actualizacion 14/10/2026: Escala 100 + 10 z en 16/18 (documento tecnico, seccion 4); interpretabilidad por ablacion y permutacion, sin SHAP (seccion 8).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Video del entregable 4: grabacion automatizada con narracion y subtitulos
Graba el recorrido del dashboard con Playwright segun el guion corto (20 segmentos en
video/narracion.json), parte la narracion de ElevenLabs por pausas (video/partir_voz.py),
recorta los huecos de recalculo y quema subtitulos. Resultado: 4:12 a 1080p.
README, guia (seccion 43) y bitacora actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bitacora_Modelado_ISAC.xlsx
+++ b/Bitacora_Modelado_ISAC.xlsx
@@ -383,7 +383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="14" min="1" max="1"/>
@@ -4757,6 +4757,46 @@
       <c r="L72" s="1" t="inlineStr">
         <is>
           <t>guia 42.5, 42.10; 24_arsenal_contraste.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>video/grabar_video.py; video/partir_voz.py; video/narracion.json</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Video del entregable 4</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>¿Se puede grabar el video sincronizado con la narración y dentro de 5:00?</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Voz sintética del sistema vs voz de ElevenLabs partida por pausas; huecos de recálculo recortados</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Video de 4:12 a 1080p con subtítulos; cifras en pantalla iguales al guion</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Cocientes de duración por segmento 0.91-1.10; 22 s de espera recortados</t>
         </is>
       </c>
     </row>
@@ -4782,7 +4822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="14" min="1" max="1"/>
@@ -5559,6 +5599,38 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>9.995</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Video del entregable 4</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>video/</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Grabar el recorrido del dashboard con narración y subtítulos</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Cerrado</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Video listo para subir a Drive (entrega 22/10)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="E2:E50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>